<commit_message>
Guía: cómo igualar la carpeta a main si falta un archivo; ruta del proyecto sin usuario fijo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TpUWhvS2qt92kuemMLkUW7
</commit_message>
<xml_diff>
--- a/docs/pruebas/registro-pruebas.xlsx
+++ b/docs/pruebas/registro-pruebas.xlsx
@@ -3806,7 +3806,7 @@
       <c r="F70" s="5" t="inlineStr">
         <is>
           <t>(F1, LAMBDA; nuevo). En PowerShell, en la carpeta del proyecto:
-` cd "C:\Users\danal\Documents\Proyectos Claude\riesgo-montecarlo-v2" npm run scan -- "RUTA\DEL\LIBRO.xlsx" `
+` cd "$HOME\Documents\Proyectos Claude\riesgo-montecarlo-v2" npm run scan -- "RUTA\DEL\LIBRO.xlsx" `
 (cambia RUTA\DEL\LIBRO.xlsx por la ruta de verdad, entre comillas; puedes poner varios libros seguidos). Hazlo con el de humedales y con los libros que pienses simular de verdad. Pásame el informe que sale en pantalla: dice qué funciones faltan (por ejemplo LAMBDA, DESREF con desplazamientos calculados o INDIRECTO) y así desarrollo solo lo que tus libros usan.</t>
         </is>
       </c>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>(F1 del plan, nuevo). Necesita Excel 365 (LAMBDA no existe en Excel 2019 ni antes). Abre, desde la carpeta del proyecto, tests\fixtures\fidelidad-lambda.xlsx (ruta completa: C:\Users\danal\Documents\Proyectos Claude\riesgo-montecarlo-v2\tests\fixtures\fidelidad-lambda.xlsx). Si Excel pregunta por habilitar la edición, sí.
+          <t>(F1 del plan, nuevo). Necesita Excel 365 (LAMBDA no existe en Excel 2019 ni antes). Abre, desde la carpeta del proyecto, tests\fixtures\fidelidad-lambda.xlsx (en la carpeta del proyecto: tests\fixtures\fidelidad-lambda.xlsx). Si Excel pregunta por habilitar la edición, sí.
 - Fórmulas → Administrador de nombres: 11 nombres. R_GAS (una constante), TC_CO2, PC_CO2, W_CO2 (celdas) y siete LAMBDA: PR_KAPPA, PR_ALFA, PR_A, PR_B, PR_P (la presión), PR_Z y FACTREC (un factorial recursivo, para ver que el motor lo manda al compatible).
 - Hoja «Fidelidad»: la columna E es lo que calcula Excel y la F, lo que calculé en Python sin Excel. Tienen que coincidir en todas las filas con «Python: …» (L-013, la presión: 40,286). L-020 y L-021 deberían dar #¡VALOR! y L-022 #¡CALC!: anota lo que salga, sea lo que sea. Si alguna celda da #¿NOMBRE?, dímelo con captura: sería que Excel no reconoció la LAMBDA tal como la escribí en el archivo.
 - Hoja «PengRobinson»: B11, B12 y B13 son la misma presión calculada con una LAMBDA con nombre, con una LAMBDA dentro de LET y con una LAMBDA invocada en la celda. Las tres, 40,286 (como la columna C). B14 (Z), 0,782; B15 (gas ideal), 51,55; B16, −21,8 %.

</xml_diff>